<commit_message>
Sept 4 inventory: 7 new pounds (Airheadz, Zlushuie, Donniesburger, Gashouse, GMO Cookies, Purple Zots, Warheadz) + deploy handoff docs
</commit_message>
<xml_diff>
--- a/Inventory/belgium420-inventory.xlsx
+++ b/Inventory/belgium420-inventory.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4667" uniqueCount="545">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5104" uniqueCount="573">
   <si>
     <t>Belgium420 inventory log</t>
   </si>
@@ -81,7 +81,7 @@
     <t>Photo files</t>
   </si>
   <si>
-    <t>Live Type chips: All 99 / Indica 13 / Hybrid 43 / Sativa 5 / Branded 34. Gap = 4 (mushrooms only).</t>
+    <t>Live Type chips: All 106 / Indica 13 / Hybrid 44 / Sativa 5 / Branded 40. Gap = 4 (mushrooms only).</t>
   </si>
   <si>
     <t>Batch</t>
@@ -1536,13 +1536,13 @@
     <t>B420-2026-2302</t>
   </si>
   <si>
-    <t>Blaze Eros · 1g Pre-roll</t>
+    <t>Blaze Eros</t>
   </si>
   <si>
     <t>Pre-roll · 1g</t>
   </si>
   <si>
-    <t>Blaze preroll lines sell indica, hybrid, and sativa flavors. One Type would be inaccurate.</t>
+    <t>Brand/flavor line — Type filter: Branded (indica, hybrid, or sativa by flavor).</t>
   </si>
   <si>
     <t>/inventory/prerolls/blaze-eros-1g-preroll-10.jpg</t>
@@ -1551,10 +1551,7 @@
     <t>B420-2026-2303</t>
   </si>
   <si>
-    <t>Heady Head · 1g Pre-roll</t>
-  </si>
-  <si>
-    <t>Heady Heads is a preroll brand with indica and hybrid SKUs by strain. Catalog name has no cultivar.</t>
+    <t>Heady Head</t>
   </si>
   <si>
     <t>/inventory/prerolls/heady-head-1g-preroll-15.jpeg</t>
@@ -1612,6 +1609,93 @@
   </si>
   <si>
     <t>/inventory/_internal/noboof-headband-hp-p-only.jpg</t>
+  </si>
+  <si>
+    <t>B420-2026-2401</t>
+  </si>
+  <si>
+    <t>Airheadz · Zip</t>
+  </si>
+  <si>
+    <t>$100.00</t>
+  </si>
+  <si>
+    <t>Premium Flower · 28g (Zip)</t>
+  </si>
+  <si>
+    <t>https://www.leafly.com/strains/airheadz</t>
+  </si>
+  <si>
+    <t>/inventory/pounds/Airheadz-100-zip.jpeg</t>
+  </si>
+  <si>
+    <t>B420-2026-2402</t>
+  </si>
+  <si>
+    <t>Zlushuie · Zip</t>
+  </si>
+  <si>
+    <t>$250.00</t>
+  </si>
+  <si>
+    <t>unmatched</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>/inventory/pounds/Zlushuie-250-zip.jpeg</t>
+  </si>
+  <si>
+    <t>B420-2026-2403</t>
+  </si>
+  <si>
+    <t>Donniesburger · Pound</t>
+  </si>
+  <si>
+    <t>/inventory/pounds/Donniesburger-850-pound.jpeg</t>
+  </si>
+  <si>
+    <t>B420-2026-2404</t>
+  </si>
+  <si>
+    <t>Gashouse · Pound</t>
+  </si>
+  <si>
+    <t>$675.00</t>
+  </si>
+  <si>
+    <t>/inventory/pounds/gashouse-675-pound.jpeg</t>
+  </si>
+  <si>
+    <t>B420-2026-2405</t>
+  </si>
+  <si>
+    <t>GMO Cookies · Pound</t>
+  </si>
+  <si>
+    <t>/inventory/pounds/GMOCookies-650-pound.jpeg</t>
+  </si>
+  <si>
+    <t>B420-2026-2406</t>
+  </si>
+  <si>
+    <t>Purple Zots · Pound</t>
+  </si>
+  <si>
+    <t>/inventory/pounds/purplezots-1200-pound.jpeg</t>
+  </si>
+  <si>
+    <t>B420-2026-2407</t>
+  </si>
+  <si>
+    <t>Warheadz · Pound</t>
+  </si>
+  <si>
+    <t>$1,875.00</t>
+  </si>
+  <si>
+    <t>/inventory/pounds/warheadz-1875-pound.jpeg</t>
   </si>
   <si>
     <t>Status</t>
@@ -1694,7 +1778,7 @@
       <color rgb="FF050505"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1741,6 +1825,11 @@
         <fgColor rgb="FFF8CBAD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4C7C3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1754,7 +1843,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1786,6 +1875,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2162,7 +2254,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2170,7 +2262,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -2178,7 +2270,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2202,7 +2294,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -2218,7 +2310,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -2226,7 +2318,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -2266,7 +2358,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -2274,7 +2366,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>108</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2509,10 +2601,10 @@
         <v>57</v>
       </c>
       <c r="M4" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="N4" s="8" t="s">
         <v>510</v>
-      </c>
-      <c r="N4" s="8" t="s">
-        <v>511</v>
       </c>
       <c r="O4" s="8" t="s">
         <v>48</v>
@@ -2530,7 +2622,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2599,6 +2691,256 @@
         <v>35</v>
       </c>
     </row>
+    <row r="2" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>535</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>536</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P2" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P3" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>544</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>546</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P4" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>551</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>552</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>553</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>554</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>555</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>556</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K6" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>557</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P6" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2608,7 +2950,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="64" customWidth="1"/>
@@ -2616,48 +2958,48 @@
     <col min="3" max="3" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="15" t="s">
-        <v>530</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>531</v>
+      <c r="B1" s="16" t="s">
+        <v>558</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B3" t="s">
         <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B4" t="s">
         <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2915,10 +3257,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>532</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>533</v>
+        <v>560</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C28" t="s">
         <v>49</v>
@@ -3047,10 +3389,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>534</v>
-      </c>
-      <c r="B40" s="16" t="s">
-        <v>533</v>
+        <v>562</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C40" t="s">
         <v>49</v>
@@ -3058,10 +3400,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>535</v>
-      </c>
-      <c r="B41" s="16" t="s">
-        <v>533</v>
+        <v>563</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C41" t="s">
         <v>49</v>
@@ -3086,7 +3428,7 @@
         <v>48</v>
       </c>
       <c r="C43" t="s">
-        <v>536</v>
+        <v>564</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -3113,10 +3455,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>537</v>
-      </c>
-      <c r="B46" s="16" t="s">
-        <v>533</v>
+        <v>565</v>
+      </c>
+      <c r="B46" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C46" t="s">
         <v>49</v>
@@ -3124,694 +3466,771 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>356</v>
+        <v>534</v>
       </c>
       <c r="B47" t="s">
         <v>48</v>
       </c>
       <c r="C47" t="s">
-        <v>355</v>
+        <v>530</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>295</v>
+        <v>543</v>
       </c>
       <c r="B48" t="s">
         <v>48</v>
       </c>
       <c r="C48" t="s">
-        <v>291</v>
+        <v>542</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>271</v>
+        <v>550</v>
       </c>
       <c r="B49" t="s">
         <v>48</v>
       </c>
       <c r="C49" t="s">
-        <v>267</v>
+        <v>549</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>237</v>
+        <v>356</v>
       </c>
       <c r="B50" t="s">
         <v>48</v>
       </c>
       <c r="C50" t="s">
-        <v>235</v>
+        <v>355</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>538</v>
-      </c>
-      <c r="B51" s="16" t="s">
-        <v>533</v>
+        <v>540</v>
+      </c>
+      <c r="B51" t="s">
+        <v>48</v>
       </c>
       <c r="C51" t="s">
-        <v>49</v>
+        <v>536</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>408</v>
+        <v>295</v>
       </c>
       <c r="B52" t="s">
         <v>48</v>
       </c>
       <c r="C52" t="s">
-        <v>405</v>
+        <v>291</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>353</v>
+        <v>271</v>
       </c>
       <c r="B53" t="s">
         <v>48</v>
       </c>
       <c r="C53" t="s">
-        <v>349</v>
+        <v>267</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>65</v>
+        <v>237</v>
       </c>
       <c r="B54" t="s">
         <v>48</v>
       </c>
       <c r="C54" t="s">
-        <v>60</v>
+        <v>235</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>112</v>
-      </c>
-      <c r="B55" t="s">
-        <v>48</v>
+        <v>566</v>
+      </c>
+      <c r="B55" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C55" t="s">
-        <v>107</v>
+        <v>49</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>344</v>
+        <v>408</v>
       </c>
       <c r="B56" t="s">
         <v>48</v>
       </c>
       <c r="C56" t="s">
-        <v>341</v>
+        <v>405</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>339</v>
+        <v>353</v>
       </c>
       <c r="B57" t="s">
         <v>48</v>
       </c>
       <c r="C57" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>325</v>
+        <v>65</v>
       </c>
       <c r="B58" t="s">
         <v>48</v>
       </c>
       <c r="C58" t="s">
-        <v>322</v>
+        <v>60</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>79</v>
+        <v>112</v>
       </c>
       <c r="B59" t="s">
         <v>48</v>
       </c>
       <c r="C59" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>87</v>
+        <v>344</v>
       </c>
       <c r="B60" t="s">
         <v>48</v>
       </c>
       <c r="C60" t="s">
-        <v>85</v>
+        <v>341</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>250</v>
+        <v>339</v>
       </c>
       <c r="B61" t="s">
         <v>48</v>
       </c>
       <c r="C61" t="s">
-        <v>249</v>
+        <v>336</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>362</v>
+        <v>325</v>
       </c>
       <c r="B62" t="s">
         <v>48</v>
       </c>
       <c r="C62" t="s">
-        <v>358</v>
+        <v>322</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>247</v>
+        <v>79</v>
       </c>
       <c r="B63" t="s">
         <v>48</v>
       </c>
       <c r="C63" t="s">
-        <v>243</v>
+        <v>78</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>253</v>
+        <v>87</v>
       </c>
       <c r="B64" t="s">
         <v>48</v>
       </c>
       <c r="C64" t="s">
-        <v>252</v>
+        <v>85</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>373</v>
+        <v>250</v>
       </c>
       <c r="B65" t="s">
         <v>48</v>
       </c>
       <c r="C65" t="s">
-        <v>369</v>
+        <v>249</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>307</v>
+        <v>362</v>
       </c>
       <c r="B66" t="s">
         <v>48</v>
       </c>
       <c r="C66" t="s">
-        <v>303</v>
+        <v>358</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>316</v>
+        <v>247</v>
       </c>
       <c r="B67" t="s">
         <v>48</v>
       </c>
       <c r="C67" t="s">
-        <v>314</v>
+        <v>243</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>119</v>
+        <v>253</v>
       </c>
       <c r="B68" t="s">
         <v>48</v>
       </c>
       <c r="C68" t="s">
-        <v>114</v>
+        <v>252</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>301</v>
+        <v>373</v>
       </c>
       <c r="B69" t="s">
         <v>48</v>
       </c>
       <c r="C69" t="s">
-        <v>297</v>
+        <v>369</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>58</v>
+        <v>307</v>
       </c>
       <c r="B70" t="s">
         <v>48</v>
       </c>
       <c r="C70" t="s">
-        <v>51</v>
+        <v>303</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>233</v>
+        <v>316</v>
       </c>
       <c r="B71" t="s">
         <v>48</v>
       </c>
       <c r="C71" t="s">
-        <v>231</v>
+        <v>314</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B72" t="s">
         <v>48</v>
       </c>
       <c r="C72" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>91</v>
+        <v>547</v>
       </c>
       <c r="B73" t="s">
         <v>48</v>
       </c>
       <c r="C73" t="s">
-        <v>89</v>
+        <v>545</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>539</v>
-      </c>
-      <c r="B74" s="16" t="s">
-        <v>533</v>
+        <v>301</v>
+      </c>
+      <c r="B74" t="s">
+        <v>48</v>
       </c>
       <c r="C74" t="s">
-        <v>49</v>
+        <v>297</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>540</v>
-      </c>
-      <c r="B75" s="16" t="s">
-        <v>533</v>
+        <v>58</v>
+      </c>
+      <c r="B75" t="s">
+        <v>48</v>
       </c>
       <c r="C75" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>320</v>
+        <v>233</v>
       </c>
       <c r="B76" t="s">
         <v>48</v>
       </c>
       <c r="C76" t="s">
-        <v>318</v>
+        <v>231</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>265</v>
+        <v>125</v>
       </c>
       <c r="B77" t="s">
         <v>48</v>
       </c>
       <c r="C77" t="s">
-        <v>262</v>
+        <v>121</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>289</v>
+        <v>91</v>
       </c>
       <c r="B78" t="s">
         <v>48</v>
       </c>
       <c r="C78" t="s">
-        <v>287</v>
+        <v>89</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>76</v>
-      </c>
-      <c r="B79" t="s">
-        <v>48</v>
+        <v>567</v>
+      </c>
+      <c r="B79" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C79" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>105</v>
-      </c>
-      <c r="B80" t="s">
-        <v>48</v>
+        <v>568</v>
+      </c>
+      <c r="B80" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C80" t="s">
-        <v>101</v>
+        <v>49</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>541</v>
-      </c>
-      <c r="B81" s="16" t="s">
-        <v>533</v>
+        <v>320</v>
+      </c>
+      <c r="B81" t="s">
+        <v>48</v>
       </c>
       <c r="C81" t="s">
-        <v>49</v>
+        <v>318</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>347</v>
+        <v>265</v>
       </c>
       <c r="B82" t="s">
         <v>48</v>
       </c>
       <c r="C82" t="s">
-        <v>346</v>
+        <v>262</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>542</v>
-      </c>
-      <c r="B83" s="16" t="s">
-        <v>533</v>
+        <v>289</v>
+      </c>
+      <c r="B83" t="s">
+        <v>48</v>
       </c>
       <c r="C83" t="s">
-        <v>49</v>
+        <v>287</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>330</v>
+        <v>76</v>
       </c>
       <c r="B84" t="s">
         <v>48</v>
       </c>
       <c r="C84" t="s">
-        <v>327</v>
+        <v>71</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>256</v>
+        <v>105</v>
       </c>
       <c r="B85" t="s">
         <v>48</v>
       </c>
       <c r="C85" t="s">
-        <v>255</v>
+        <v>101</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>69</v>
-      </c>
-      <c r="B86" t="s">
-        <v>48</v>
+        <v>569</v>
+      </c>
+      <c r="B86" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C86" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>543</v>
-      </c>
-      <c r="B87" s="16" t="s">
-        <v>533</v>
+        <v>347</v>
+      </c>
+      <c r="B87" t="s">
+        <v>48</v>
       </c>
       <c r="C87" t="s">
-        <v>49</v>
+        <v>346</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>312</v>
-      </c>
-      <c r="B88" t="s">
-        <v>48</v>
+        <v>570</v>
+      </c>
+      <c r="B88" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C88" t="s">
-        <v>309</v>
+        <v>49</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>47</v>
+        <v>330</v>
       </c>
       <c r="B89" t="s">
         <v>48</v>
       </c>
       <c r="C89" t="s">
-        <v>37</v>
+        <v>327</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>131</v>
+        <v>553</v>
       </c>
       <c r="B90" t="s">
         <v>48</v>
       </c>
       <c r="C90" t="s">
-        <v>127</v>
+        <v>552</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="B91" t="s">
         <v>48</v>
       </c>
       <c r="C91" t="s">
-        <v>239</v>
+        <v>255</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>544</v>
-      </c>
-      <c r="B92" s="16" t="s">
-        <v>533</v>
+        <v>69</v>
+      </c>
+      <c r="B92" t="s">
+        <v>48</v>
       </c>
       <c r="C92" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>280</v>
-      </c>
-      <c r="B93" t="s">
-        <v>48</v>
+        <v>571</v>
+      </c>
+      <c r="B93" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C93" t="s">
-        <v>276</v>
+        <v>49</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>274</v>
+        <v>312</v>
       </c>
       <c r="B94" t="s">
         <v>48</v>
       </c>
       <c r="C94" t="s">
-        <v>273</v>
+        <v>309</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>334</v>
+        <v>47</v>
       </c>
       <c r="B95" t="s">
         <v>48</v>
       </c>
       <c r="C95" t="s">
-        <v>332</v>
+        <v>37</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>285</v>
+        <v>131</v>
       </c>
       <c r="B96" t="s">
         <v>48</v>
       </c>
       <c r="C96" t="s">
-        <v>282</v>
+        <v>127</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>99</v>
+        <v>241</v>
       </c>
       <c r="B97" t="s">
         <v>48</v>
       </c>
       <c r="C97" t="s">
-        <v>93</v>
+        <v>239</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>367</v>
-      </c>
-      <c r="B98" t="s">
-        <v>48</v>
+        <v>572</v>
+      </c>
+      <c r="B98" s="17" t="s">
+        <v>561</v>
       </c>
       <c r="C98" t="s">
-        <v>364</v>
+        <v>49</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="B99" t="s">
         <v>48</v>
       </c>
       <c r="C99" t="s">
-        <v>258</v>
+        <v>276</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>83</v>
+        <v>274</v>
       </c>
       <c r="B100" t="s">
         <v>48</v>
       </c>
       <c r="C100" t="s">
-        <v>81</v>
+        <v>273</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>507</v>
+        <v>334</v>
       </c>
       <c r="B101" t="s">
         <v>48</v>
       </c>
       <c r="C101" t="s">
-        <v>504</v>
+        <v>332</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>502</v>
+        <v>285</v>
       </c>
       <c r="B102" t="s">
         <v>48</v>
       </c>
       <c r="C102" t="s">
-        <v>497</v>
+        <v>282</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>511</v>
+        <v>99</v>
       </c>
       <c r="B103" t="s">
         <v>48</v>
       </c>
       <c r="C103" t="s">
-        <v>509</v>
+        <v>93</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>389</v>
+        <v>367</v>
       </c>
       <c r="B104" t="s">
         <v>48</v>
       </c>
       <c r="C104" t="s">
-        <v>386</v>
+        <v>364</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>394</v>
+        <v>260</v>
       </c>
       <c r="B105" t="s">
         <v>48</v>
       </c>
       <c r="C105" t="s">
-        <v>391</v>
+        <v>258</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>384</v>
+        <v>557</v>
       </c>
       <c r="B106" t="s">
         <v>48</v>
       </c>
       <c r="C106" t="s">
-        <v>380</v>
+        <v>555</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>399</v>
+        <v>83</v>
       </c>
       <c r="B107" t="s">
         <v>48</v>
       </c>
       <c r="C107" t="s">
-        <v>396</v>
+        <v>81</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>378</v>
+        <v>507</v>
       </c>
       <c r="B108" t="s">
         <v>48</v>
       </c>
       <c r="C108" t="s">
-        <v>375</v>
+        <v>504</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>502</v>
+      </c>
+      <c r="B109" t="s">
+        <v>48</v>
+      </c>
+      <c r="C109" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>510</v>
+      </c>
+      <c r="B110" t="s">
+        <v>48</v>
+      </c>
+      <c r="C110" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>389</v>
+      </c>
+      <c r="B111" t="s">
+        <v>48</v>
+      </c>
+      <c r="C111" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>394</v>
+      </c>
+      <c r="B112" t="s">
+        <v>48</v>
+      </c>
+      <c r="C112" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>384</v>
+      </c>
+      <c r="B113" t="s">
+        <v>48</v>
+      </c>
+      <c r="C113" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>399</v>
+      </c>
+      <c r="B114" t="s">
+        <v>48</v>
+      </c>
+      <c r="C114" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>378</v>
+      </c>
+      <c r="B115" t="s">
+        <v>48</v>
+      </c>
+      <c r="C115" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
         <v>403</v>
       </c>
-      <c r="B109" t="s">
-        <v>48</v>
-      </c>
-      <c r="C109" t="s">
+      <c r="B116" t="s">
+        <v>48</v>
+      </c>
+      <c r="C116" t="s">
         <v>401</v>
       </c>
     </row>
@@ -3824,7 +4243,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P100"/>
+  <dimension ref="A1:P107"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -8681,10 +9100,10 @@
         <v>57</v>
       </c>
       <c r="M97" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="N97" s="8" t="s">
         <v>510</v>
-      </c>
-      <c r="N97" s="8" t="s">
-        <v>511</v>
       </c>
       <c r="O97" s="8" t="s">
         <v>48</v>
@@ -8695,28 +9114,28 @@
     </row>
     <row r="98" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="8" t="s">
+        <v>511</v>
+      </c>
+      <c r="B98" s="8" t="s">
         <v>512</v>
       </c>
-      <c r="B98" s="8" t="s">
+      <c r="C98" s="8" t="s">
         <v>513</v>
-      </c>
-      <c r="C98" s="8" t="s">
-        <v>514</v>
       </c>
       <c r="D98" s="8" t="s">
         <v>39</v>
       </c>
       <c r="E98" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F98" s="8" t="s">
         <v>283</v>
       </c>
       <c r="G98" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="H98" s="9" t="s">
         <v>516</v>
-      </c>
-      <c r="H98" s="9" t="s">
-        <v>517</v>
       </c>
       <c r="I98" s="8" t="s">
         <v>41</v>
@@ -8734,7 +9153,7 @@
         <v>49</v>
       </c>
       <c r="N98" s="8" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="O98" s="8" t="s">
         <v>48</v>
@@ -8745,19 +9164,19 @@
     </row>
     <row r="99" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
+        <v>518</v>
+      </c>
+      <c r="B99" s="8" t="s">
         <v>519</v>
       </c>
-      <c r="B99" s="8" t="s">
-        <v>520</v>
-      </c>
       <c r="C99" s="8" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D99" s="8" t="s">
         <v>39</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F99" s="8" t="s">
         <v>41</v>
@@ -8766,13 +9185,13 @@
         <v>130</v>
       </c>
       <c r="H99" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="I99" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J99" s="8" t="s">
         <v>521</v>
-      </c>
-      <c r="I99" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="J99" s="8" t="s">
-        <v>522</v>
       </c>
       <c r="K99" s="11" t="s">
         <v>56</v>
@@ -8781,10 +9200,10 @@
         <v>57</v>
       </c>
       <c r="M99" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="N99" s="8" t="s">
         <v>523</v>
-      </c>
-      <c r="N99" s="8" t="s">
-        <v>524</v>
       </c>
       <c r="O99" s="8" t="s">
         <v>48</v>
@@ -8795,28 +9214,28 @@
     </row>
     <row r="100" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="B100" s="8" t="s">
         <v>525</v>
       </c>
-      <c r="B100" s="8" t="s">
-        <v>526</v>
-      </c>
       <c r="C100" s="8" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D100" s="8" t="s">
         <v>39</v>
       </c>
       <c r="E100" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F100" s="8" t="s">
         <v>283</v>
       </c>
       <c r="G100" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="H100" s="9" t="s">
         <v>527</v>
-      </c>
-      <c r="H100" s="9" t="s">
-        <v>528</v>
       </c>
       <c r="I100" s="8" t="s">
         <v>41</v>
@@ -8834,13 +9253,363 @@
         <v>49</v>
       </c>
       <c r="N100" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="O100" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P100" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="101" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="8" t="s">
         <v>529</v>
       </c>
-      <c r="O100" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="P100" s="8" t="s">
-        <v>48</v>
+      <c r="B101" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C101" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="D101" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E101" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="F101" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G101" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="H101" s="9" t="s">
+        <v>533</v>
+      </c>
+      <c r="I101" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J101" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="K101" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L101" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M101" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N101" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="O101" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P101" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="102" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="8" t="s">
+        <v>535</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>536</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="D102" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E102" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="F102" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G102" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H102" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I102" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J102" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K102" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L102" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M102" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N102" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="O102" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P102" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="103" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="B103" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="C103" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D103" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E103" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F103" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G103" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H103" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I103" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J103" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K103" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L103" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M103" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N103" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="O103" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P103" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="104" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="8" t="s">
+        <v>544</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>546</v>
+      </c>
+      <c r="D104" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E104" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F104" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G104" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H104" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I104" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J104" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K104" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L104" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M104" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N104" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="O104" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P104" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="105" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="8" t="s">
+        <v>548</v>
+      </c>
+      <c r="B105" s="8" t="s">
+        <v>549</v>
+      </c>
+      <c r="C105" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D105" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E105" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F105" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G105" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="H105" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="I105" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J105" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="K105" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L105" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M105" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N105" s="8" t="s">
+        <v>550</v>
+      </c>
+      <c r="O105" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P105" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="8" t="s">
+        <v>551</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>552</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D106" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E106" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G106" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H106" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I106" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J106" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K106" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L106" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M106" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N106" s="8" t="s">
+        <v>553</v>
+      </c>
+      <c r="O106" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P106" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="107" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="8" t="s">
+        <v>554</v>
+      </c>
+      <c r="B107" s="8" t="s">
+        <v>555</v>
+      </c>
+      <c r="C107" s="8" t="s">
+        <v>556</v>
+      </c>
+      <c r="D107" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E107" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F107" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G107" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H107" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I107" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J107" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K107" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L107" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M107" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N107" s="8" t="s">
+        <v>557</v>
+      </c>
+      <c r="O107" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P107" s="8" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -8898,6 +9667,8 @@
     <hyperlink ref="H98" r:id="rId50"/>
     <hyperlink ref="H99" r:id="rId51"/>
     <hyperlink ref="H100" r:id="rId52"/>
+    <hyperlink ref="H101" r:id="rId53"/>
+    <hyperlink ref="H105" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -8906,7 +9677,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P60"/>
+  <dimension ref="A1:P67"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -11777,28 +12548,28 @@
     </row>
     <row r="58" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
+        <v>511</v>
+      </c>
+      <c r="B58" s="8" t="s">
         <v>512</v>
       </c>
-      <c r="B58" s="8" t="s">
+      <c r="C58" s="8" t="s">
         <v>513</v>
-      </c>
-      <c r="C58" s="8" t="s">
-        <v>514</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>39</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F58" s="8" t="s">
         <v>283</v>
       </c>
       <c r="G58" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="H58" s="9" t="s">
         <v>516</v>
-      </c>
-      <c r="H58" s="9" t="s">
-        <v>517</v>
       </c>
       <c r="I58" s="8" t="s">
         <v>41</v>
@@ -11816,7 +12587,7 @@
         <v>49</v>
       </c>
       <c r="N58" s="8" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="O58" s="8" t="s">
         <v>48</v>
@@ -11827,19 +12598,19 @@
     </row>
     <row r="59" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
+        <v>518</v>
+      </c>
+      <c r="B59" s="8" t="s">
         <v>519</v>
       </c>
-      <c r="B59" s="8" t="s">
-        <v>520</v>
-      </c>
       <c r="C59" s="8" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>39</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F59" s="8" t="s">
         <v>41</v>
@@ -11848,13 +12619,13 @@
         <v>130</v>
       </c>
       <c r="H59" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="I59" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J59" s="8" t="s">
         <v>521</v>
-      </c>
-      <c r="I59" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="J59" s="8" t="s">
-        <v>522</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>56</v>
@@ -11863,10 +12634,10 @@
         <v>57</v>
       </c>
       <c r="M59" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="N59" s="8" t="s">
         <v>523</v>
-      </c>
-      <c r="N59" s="8" t="s">
-        <v>524</v>
       </c>
       <c r="O59" s="8" t="s">
         <v>48</v>
@@ -11877,28 +12648,28 @@
     </row>
     <row r="60" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="B60" s="8" t="s">
         <v>525</v>
       </c>
-      <c r="B60" s="8" t="s">
-        <v>526</v>
-      </c>
       <c r="C60" s="8" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>39</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F60" s="8" t="s">
         <v>283</v>
       </c>
       <c r="G60" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="H60" s="9" t="s">
         <v>527</v>
-      </c>
-      <c r="H60" s="9" t="s">
-        <v>528</v>
       </c>
       <c r="I60" s="8" t="s">
         <v>41</v>
@@ -11916,13 +12687,363 @@
         <v>49</v>
       </c>
       <c r="N60" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="O60" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P60" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="8" t="s">
         <v>529</v>
       </c>
-      <c r="O60" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="P60" s="8" t="s">
-        <v>48</v>
+      <c r="B61" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="D61" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E61" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="F61" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G61" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="H61" s="9" t="s">
+        <v>533</v>
+      </c>
+      <c r="I61" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J61" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="K61" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L61" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M61" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N61" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="O61" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P61" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="8" t="s">
+        <v>535</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>536</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="D62" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E62" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="F62" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G62" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H62" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I62" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J62" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K62" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L62" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M62" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N62" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="O62" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P62" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="C63" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D63" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E63" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F63" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G63" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H63" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I63" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J63" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K63" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L63" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M63" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N63" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="O63" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P63" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="8" t="s">
+        <v>544</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>546</v>
+      </c>
+      <c r="D64" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F64" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G64" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H64" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I64" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J64" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K64" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L64" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M64" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N64" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="O64" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P64" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="8" t="s">
+        <v>548</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>549</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D65" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E65" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F65" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G65" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="H65" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="I65" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J65" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="K65" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L65" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M65" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N65" s="8" t="s">
+        <v>550</v>
+      </c>
+      <c r="O65" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P65" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="8" t="s">
+        <v>551</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>552</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H66" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I66" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J66" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K66" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L66" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M66" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N66" s="8" t="s">
+        <v>553</v>
+      </c>
+      <c r="O66" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P66" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="8" t="s">
+        <v>554</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>555</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>556</v>
+      </c>
+      <c r="D67" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E67" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F67" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G67" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I67" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J67" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K67" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L67" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M67" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N67" s="8" t="s">
+        <v>557</v>
+      </c>
+      <c r="O67" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P67" s="8" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -11978,6 +13099,8 @@
     <hyperlink ref="H58" r:id="rId48"/>
     <hyperlink ref="H59" r:id="rId49"/>
     <hyperlink ref="H60" r:id="rId50"/>
+    <hyperlink ref="H61" r:id="rId51"/>
+    <hyperlink ref="H65" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -14034,7 +15157,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -16605,28 +17728,28 @@
     </row>
     <row r="52" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
+        <v>511</v>
+      </c>
+      <c r="B52" s="8" t="s">
         <v>512</v>
       </c>
-      <c r="B52" s="8" t="s">
+      <c r="C52" s="8" t="s">
         <v>513</v>
-      </c>
-      <c r="C52" s="8" t="s">
-        <v>514</v>
       </c>
       <c r="D52" s="8" t="s">
         <v>39</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F52" s="8" t="s">
         <v>283</v>
       </c>
       <c r="G52" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="H52" s="9" t="s">
         <v>516</v>
-      </c>
-      <c r="H52" s="9" t="s">
-        <v>517</v>
       </c>
       <c r="I52" s="8" t="s">
         <v>41</v>
@@ -16644,7 +17767,7 @@
         <v>49</v>
       </c>
       <c r="N52" s="8" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="O52" s="8" t="s">
         <v>48</v>
@@ -16655,19 +17778,19 @@
     </row>
     <row r="53" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
+        <v>518</v>
+      </c>
+      <c r="B53" s="8" t="s">
         <v>519</v>
       </c>
-      <c r="B53" s="8" t="s">
-        <v>520</v>
-      </c>
       <c r="C53" s="8" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D53" s="8" t="s">
         <v>39</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F53" s="8" t="s">
         <v>41</v>
@@ -16676,13 +17799,13 @@
         <v>130</v>
       </c>
       <c r="H53" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="I53" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J53" s="8" t="s">
         <v>521</v>
-      </c>
-      <c r="I53" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="J53" s="8" t="s">
-        <v>522</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>56</v>
@@ -16691,10 +17814,10 @@
         <v>57</v>
       </c>
       <c r="M53" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="N53" s="8" t="s">
         <v>523</v>
-      </c>
-      <c r="N53" s="8" t="s">
-        <v>524</v>
       </c>
       <c r="O53" s="8" t="s">
         <v>48</v>
@@ -16705,28 +17828,28 @@
     </row>
     <row r="54" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="B54" s="8" t="s">
         <v>525</v>
       </c>
-      <c r="B54" s="8" t="s">
-        <v>526</v>
-      </c>
       <c r="C54" s="8" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D54" s="8" t="s">
         <v>39</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F54" s="8" t="s">
         <v>283</v>
       </c>
       <c r="G54" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="H54" s="9" t="s">
         <v>527</v>
-      </c>
-      <c r="H54" s="9" t="s">
-        <v>528</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>41</v>
@@ -16744,13 +17867,363 @@
         <v>49</v>
       </c>
       <c r="N54" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="O54" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P54" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="8" t="s">
         <v>529</v>
       </c>
-      <c r="O54" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="P54" s="8" t="s">
-        <v>48</v>
+      <c r="B55" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E55" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="F55" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G55" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="H55" s="9" t="s">
+        <v>533</v>
+      </c>
+      <c r="I55" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J55" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="K55" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L55" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M55" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N55" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="O55" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P55" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="8" t="s">
+        <v>535</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>536</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G56" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H56" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I56" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J56" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K56" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L56" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M56" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N56" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="O56" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P56" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D57" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F57" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H57" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I57" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J57" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K57" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L57" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M57" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N57" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="O57" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P57" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="8" t="s">
+        <v>544</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>546</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G58" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H58" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I58" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J58" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K58" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L58" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M58" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N58" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="O58" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P58" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="8" t="s">
+        <v>548</v>
+      </c>
+      <c r="B59" s="8" t="s">
+        <v>549</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D59" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G59" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="H59" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="I59" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J59" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="K59" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L59" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="M59" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N59" s="8" t="s">
+        <v>550</v>
+      </c>
+      <c r="O59" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P59" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="8" t="s">
+        <v>551</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>552</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D60" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F60" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G60" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H60" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I60" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J60" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K60" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L60" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M60" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N60" s="8" t="s">
+        <v>553</v>
+      </c>
+      <c r="O60" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P60" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="8" t="s">
+        <v>554</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>555</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>556</v>
+      </c>
+      <c r="D61" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E61" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F61" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G61" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H61" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I61" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J61" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K61" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="L61" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M61" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N61" s="8" t="s">
+        <v>557</v>
+      </c>
+      <c r="O61" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P61" s="8" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -16798,6 +18271,8 @@
     <hyperlink ref="H52" r:id="rId40"/>
     <hyperlink ref="H53" r:id="rId41"/>
     <hyperlink ref="H54" r:id="rId42"/>
+    <hyperlink ref="H55" r:id="rId43"/>
+    <hyperlink ref="H59" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>